<commit_message>
I don't know what actually changed with this, but it all looks normal.
</commit_message>
<xml_diff>
--- a/UW_Nest_Behavioral_Sheets_Cleaned.xlsx
+++ b/UW_Nest_Behavioral_Sheets_Cleaned.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10118"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10222"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jacobchung/coding_projects/UW_Owrasse_Behavior/Raw_UW_Behaviour_datasets/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jacobchung/coding_projects/Owrasse_Underwater_Behavioral_Sheet/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{9BE46255-CAE6-A149-923A-8062B821BDA9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{997F1C79-08CD-5947-BC14-AFC7DE4D7B69}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-11220" yWindow="-28300" windowWidth="51200" windowHeight="28300" xr2:uid="{F3336806-D2AA-0243-9E92-F92A9E05C0A5}"/>
+    <workbookView xWindow="-20" yWindow="520" windowWidth="27760" windowHeight="17500" xr2:uid="{F3336806-D2AA-0243-9E92-F92A9E05C0A5}"/>
   </bookViews>
   <sheets>
     <sheet name="UW_Behavior_Sheets" sheetId="1" r:id="rId1"/>
@@ -84,7 +84,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="896" uniqueCount="342">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="959" uniqueCount="348">
   <si>
     <t>Date</t>
   </si>
@@ -3173,6 +3173,24 @@
       <t xml:space="preserve"> preform courtship to a Female</t>
     </r>
   </si>
+  <si>
+    <t>Focus?</t>
+  </si>
+  <si>
+    <t>No</t>
+  </si>
+  <si>
+    <t>Yes</t>
+  </si>
+  <si>
+    <t>By assoiation</t>
+  </si>
+  <si>
+    <t>Possibly</t>
+  </si>
+  <si>
+    <t>By Association</t>
+  </si>
 </sst>
 </file>
 
@@ -3301,7 +3319,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="12">
+  <fills count="16">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -3365,6 +3383,30 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFF4F482"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF0000"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -3797,9 +3839,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="138">
+  <cellXfs count="142">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="20" fontId="0" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="20" fontId="3" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -3839,11 +3881,11 @@
     <xf numFmtId="20" fontId="0" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="14" fontId="0" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
@@ -3871,16 +3913,16 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="9" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="10" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment textRotation="90"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment textRotation="90"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="5" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -3990,18 +4032,22 @@
     <xf numFmtId="0" fontId="1" fillId="7" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="7" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="7" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="8" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="7" fillId="6" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="7" fillId="7" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="7" fillId="7" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="7" fillId="6" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="7" fillId="9" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="7" fillId="7" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="7" fillId="8" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="6" fillId="11" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="6" fillId="10" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="9" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="11" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="10" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -34655,14 +34701,14 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CD62DE66-DE7D-D74F-8048-74B8D7966E23}">
-  <dimension ref="A1:G76"/>
+  <dimension ref="A1:H76"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="46.6640625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="54.1640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A1" s="136" t="s">
         <v>271</v>
       </c>
@@ -34670,7 +34716,7 @@
         <v>272</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A2" s="136" t="s">
         <v>94</v>
       </c>
@@ -34678,7 +34724,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A3" s="136" t="s">
         <v>270</v>
       </c>
@@ -34689,7 +34735,7 @@
         <v>268</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A4" s="136" t="s">
         <v>273</v>
       </c>
@@ -34700,7 +34746,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A5" s="136" t="s">
         <v>274</v>
       </c>
@@ -34708,7 +34754,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A6" s="136" t="s">
         <v>275</v>
       </c>
@@ -34716,7 +34762,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A7" s="136" t="s">
         <v>277</v>
       </c>
@@ -34724,7 +34770,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A8" s="136" t="s">
         <v>276</v>
       </c>
@@ -34732,508 +34778,821 @@
         <v>98</v>
       </c>
     </row>
-    <row r="14" spans="1:7" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:8" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A14" s="137" t="s">
         <v>278</v>
       </c>
       <c r="B14" s="137" t="s">
         <v>279</v>
       </c>
+      <c r="H14" s="137" t="s">
+        <v>342</v>
+      </c>
     </row>
-    <row r="15" spans="1:7" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:8" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A15" s="126" t="s">
         <v>8</v>
       </c>
       <c r="B15" t="s">
         <v>280</v>
       </c>
+      <c r="F15" s="138"/>
+      <c r="G15" s="138"/>
+      <c r="H15" s="138" t="s">
+        <v>344</v>
+      </c>
     </row>
-    <row r="16" spans="1:7" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:8" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A16" s="127" t="s">
         <v>9</v>
       </c>
       <c r="B16" t="s">
         <v>281</v>
       </c>
+      <c r="F16" s="139"/>
+      <c r="G16" s="139"/>
+      <c r="H16" s="139" t="s">
+        <v>343</v>
+      </c>
     </row>
-    <row r="17" spans="1:2" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:8" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A17" s="127" t="s">
         <v>10</v>
       </c>
       <c r="B17" t="s">
         <v>282</v>
       </c>
+      <c r="F17" s="139"/>
+      <c r="G17" s="139"/>
+      <c r="H17" s="139" t="s">
+        <v>343</v>
+      </c>
     </row>
-    <row r="18" spans="1:2" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:8" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A18" s="127" t="s">
         <v>11</v>
       </c>
       <c r="B18" t="s">
         <v>283</v>
       </c>
+      <c r="F18" s="139"/>
+      <c r="G18" s="139"/>
+      <c r="H18" s="139" t="s">
+        <v>343</v>
+      </c>
     </row>
-    <row r="19" spans="1:2" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:8" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A19" s="128" t="s">
         <v>12</v>
       </c>
       <c r="B19" t="s">
         <v>284</v>
       </c>
+      <c r="F19" s="139"/>
+      <c r="G19" s="139"/>
+      <c r="H19" s="139" t="s">
+        <v>343</v>
+      </c>
     </row>
-    <row r="20" spans="1:2" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:8" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A20" s="129" t="s">
         <v>13</v>
       </c>
       <c r="B20" t="s">
         <v>285</v>
       </c>
+      <c r="F20" s="139"/>
+      <c r="G20" s="139"/>
+      <c r="H20" s="139" t="s">
+        <v>343</v>
+      </c>
     </row>
-    <row r="21" spans="1:2" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:8" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A21" s="130" t="s">
         <v>14</v>
       </c>
       <c r="B21" t="s">
         <v>286</v>
       </c>
+      <c r="F21" s="138"/>
+      <c r="G21" s="138"/>
+      <c r="H21" s="138" t="s">
+        <v>344</v>
+      </c>
     </row>
-    <row r="22" spans="1:2" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:8" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A22" s="131" t="s">
         <v>18</v>
       </c>
       <c r="B22" t="s">
         <v>287</v>
       </c>
+      <c r="F22" s="138"/>
+      <c r="G22" s="138"/>
+      <c r="H22" s="138" t="s">
+        <v>344</v>
+      </c>
     </row>
-    <row r="23" spans="1:2" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:8" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A23" s="132" t="s">
         <v>15</v>
       </c>
       <c r="B23" s="5" t="s">
         <v>288</v>
       </c>
+      <c r="F23" s="138"/>
+      <c r="G23" s="138"/>
+      <c r="H23" s="138" t="s">
+        <v>344</v>
+      </c>
     </row>
-    <row r="24" spans="1:2" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:8" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A24" s="133" t="s">
         <v>16</v>
       </c>
       <c r="B24" s="5" t="s">
         <v>289</v>
       </c>
+      <c r="F24" s="138"/>
+      <c r="G24" s="138"/>
+      <c r="H24" s="138" t="s">
+        <v>344</v>
+      </c>
     </row>
-    <row r="25" spans="1:2" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:8" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A25" s="130" t="s">
         <v>19</v>
       </c>
       <c r="B25" t="s">
         <v>290</v>
       </c>
+      <c r="F25" s="138"/>
+      <c r="G25" s="138"/>
+      <c r="H25" s="138" t="s">
+        <v>344</v>
+      </c>
     </row>
-    <row r="26" spans="1:2" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:8" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A26" s="131" t="s">
         <v>17</v>
       </c>
       <c r="B26" t="s">
         <v>291</v>
       </c>
+      <c r="F26" s="138"/>
+      <c r="G26" s="138"/>
+      <c r="H26" s="138" t="s">
+        <v>344</v>
+      </c>
     </row>
-    <row r="27" spans="1:2" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:8" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A27" s="131" t="s">
         <v>20</v>
       </c>
       <c r="B27" t="s">
         <v>292</v>
       </c>
+      <c r="F27" s="138"/>
+      <c r="G27" s="138"/>
+      <c r="H27" s="138" t="s">
+        <v>344</v>
+      </c>
     </row>
-    <row r="28" spans="1:2" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:8" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A28" s="131" t="s">
         <v>21</v>
       </c>
       <c r="B28" t="s">
         <v>293</v>
       </c>
+      <c r="F28" s="138"/>
+      <c r="G28" s="138"/>
+      <c r="H28" s="138" t="s">
+        <v>344</v>
+      </c>
     </row>
-    <row r="29" spans="1:2" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:8" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A29" s="132" t="s">
         <v>22</v>
       </c>
       <c r="B29" t="s">
         <v>294</v>
       </c>
+      <c r="F29" s="138"/>
+      <c r="G29" s="138"/>
+      <c r="H29" s="138" t="s">
+        <v>344</v>
+      </c>
     </row>
-    <row r="30" spans="1:2" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:8" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A30" s="132" t="s">
         <v>23</v>
       </c>
       <c r="B30" t="s">
         <v>295</v>
       </c>
+      <c r="F30" s="138"/>
+      <c r="G30" s="138"/>
+      <c r="H30" s="138" t="s">
+        <v>344</v>
+      </c>
     </row>
-    <row r="31" spans="1:2" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:8" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A31" s="133" t="s">
         <v>24</v>
       </c>
       <c r="B31" t="s">
         <v>296</v>
       </c>
+      <c r="F31" s="138"/>
+      <c r="G31" s="138"/>
+      <c r="H31" s="138" t="s">
+        <v>344</v>
+      </c>
     </row>
-    <row r="32" spans="1:2" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:8" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A32" s="133" t="s">
         <v>25</v>
       </c>
       <c r="B32" t="s">
         <v>297</v>
       </c>
+      <c r="F32" s="138"/>
+      <c r="G32" s="138"/>
+      <c r="H32" s="138" t="s">
+        <v>344</v>
+      </c>
     </row>
-    <row r="33" spans="1:2" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:8" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A33" s="130" t="s">
         <v>26</v>
       </c>
       <c r="B33" t="s">
         <v>298</v>
       </c>
+      <c r="F33" s="138"/>
+      <c r="G33" s="138"/>
+      <c r="H33" s="138" t="s">
+        <v>344</v>
+      </c>
     </row>
-    <row r="34" spans="1:2" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:8" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A34" s="131" t="s">
         <v>27</v>
       </c>
       <c r="B34" t="s">
         <v>299</v>
       </c>
+      <c r="F34" s="138"/>
+      <c r="G34" s="138"/>
+      <c r="H34" s="138" t="s">
+        <v>344</v>
+      </c>
     </row>
-    <row r="35" spans="1:2" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:8" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A35" s="131" t="s">
         <v>28</v>
       </c>
       <c r="B35" t="s">
         <v>300</v>
       </c>
+      <c r="F35" s="138"/>
+      <c r="G35" s="138"/>
+      <c r="H35" s="138" t="s">
+        <v>344</v>
+      </c>
     </row>
-    <row r="36" spans="1:2" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:8" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A36" s="131" t="s">
         <v>29</v>
       </c>
       <c r="B36" t="s">
         <v>301</v>
       </c>
+      <c r="F36" s="138"/>
+      <c r="G36" s="138"/>
+      <c r="H36" s="138" t="s">
+        <v>344</v>
+      </c>
     </row>
-    <row r="37" spans="1:2" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:8" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A37" s="132" t="s">
         <v>30</v>
       </c>
       <c r="B37" t="s">
         <v>302</v>
       </c>
+      <c r="F37" s="138"/>
+      <c r="G37" s="138"/>
+      <c r="H37" s="138" t="s">
+        <v>344</v>
+      </c>
     </row>
-    <row r="38" spans="1:2" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:8" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A38" s="132" t="s">
         <v>31</v>
       </c>
       <c r="B38" s="5" t="s">
         <v>303</v>
       </c>
+      <c r="F38" s="138"/>
+      <c r="G38" s="138"/>
+      <c r="H38" s="138" t="s">
+        <v>344</v>
+      </c>
     </row>
-    <row r="39" spans="1:2" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:8" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A39" s="133" t="s">
         <v>32</v>
       </c>
       <c r="B39" t="s">
         <v>304</v>
       </c>
+      <c r="F39" s="138"/>
+      <c r="G39" s="138"/>
+      <c r="H39" s="138" t="s">
+        <v>344</v>
+      </c>
     </row>
-    <row r="40" spans="1:2" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:8" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A40" s="133" t="s">
         <v>33</v>
       </c>
       <c r="B40" t="s">
         <v>305</v>
       </c>
+      <c r="F40" s="138"/>
+      <c r="G40" s="138"/>
+      <c r="H40" s="138" t="s">
+        <v>344</v>
+      </c>
     </row>
-    <row r="41" spans="1:2" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:8" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A41" s="134" t="s">
         <v>34</v>
       </c>
       <c r="B41" t="s">
         <v>307</v>
       </c>
+      <c r="F41" s="138"/>
+      <c r="G41" s="138"/>
+      <c r="H41" s="138" t="s">
+        <v>344</v>
+      </c>
     </row>
-    <row r="42" spans="1:2" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:8" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A42" s="134" t="s">
         <v>35</v>
       </c>
       <c r="B42" t="s">
         <v>306</v>
       </c>
+      <c r="F42" s="138"/>
+      <c r="G42" s="138"/>
+      <c r="H42" s="138" t="s">
+        <v>344</v>
+      </c>
     </row>
-    <row r="43" spans="1:2" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:8" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A43" s="134" t="s">
         <v>36</v>
       </c>
       <c r="B43" t="s">
         <v>308</v>
       </c>
+      <c r="F43" s="138"/>
+      <c r="G43" s="138"/>
+      <c r="H43" s="138" t="s">
+        <v>344</v>
+      </c>
     </row>
-    <row r="44" spans="1:2" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:8" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A44" s="130" t="s">
         <v>37</v>
       </c>
       <c r="B44" t="s">
         <v>309</v>
       </c>
+      <c r="F44" s="141"/>
+      <c r="G44" s="141"/>
+      <c r="H44" s="141" t="s">
+        <v>345</v>
+      </c>
     </row>
-    <row r="45" spans="1:2" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:8" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A45" s="130" t="s">
         <v>38</v>
       </c>
       <c r="B45" t="s">
         <v>310</v>
       </c>
+      <c r="F45" s="141"/>
+      <c r="G45" s="141"/>
+      <c r="H45" s="141" t="s">
+        <v>345</v>
+      </c>
     </row>
-    <row r="46" spans="1:2" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:8" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A46" s="130" t="s">
         <v>39</v>
       </c>
       <c r="B46" t="s">
         <v>311</v>
       </c>
+      <c r="F46" s="141"/>
+      <c r="G46" s="141"/>
+      <c r="H46" s="141" t="s">
+        <v>345</v>
+      </c>
     </row>
-    <row r="47" spans="1:2" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:8" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A47" s="135" t="s">
         <v>46</v>
       </c>
       <c r="B47" t="s">
         <v>312</v>
       </c>
+      <c r="F47" s="139"/>
+      <c r="G47" s="139"/>
+      <c r="H47" s="139" t="s">
+        <v>343</v>
+      </c>
     </row>
-    <row r="48" spans="1:2" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:8" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A48" s="132" t="s">
         <v>45</v>
       </c>
       <c r="B48" t="s">
         <v>313</v>
       </c>
+      <c r="F48" s="139"/>
+      <c r="G48" s="139"/>
+      <c r="H48" s="139" t="s">
+        <v>343</v>
+      </c>
     </row>
-    <row r="49" spans="1:2" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:8" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A49" s="133" t="s">
         <v>44</v>
       </c>
       <c r="B49" t="s">
         <v>314</v>
       </c>
+      <c r="F49" s="139"/>
+      <c r="G49" s="139"/>
+      <c r="H49" s="139" t="s">
+        <v>343</v>
+      </c>
     </row>
-    <row r="50" spans="1:2" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:8" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A50" s="135" t="s">
         <v>41</v>
       </c>
       <c r="B50" s="5" t="s">
         <v>315</v>
       </c>
+      <c r="F50" s="139"/>
+      <c r="G50" s="139"/>
+      <c r="H50" s="139" t="s">
+        <v>343</v>
+      </c>
     </row>
-    <row r="51" spans="1:2" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:8" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A51" s="132" t="s">
         <v>42</v>
       </c>
       <c r="B51" s="5" t="s">
         <v>316</v>
       </c>
+      <c r="F51" s="139"/>
+      <c r="G51" s="139"/>
+      <c r="H51" s="139" t="s">
+        <v>343</v>
+      </c>
     </row>
-    <row r="52" spans="1:2" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:8" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A52" s="133" t="s">
         <v>43</v>
       </c>
       <c r="B52" s="5" t="s">
         <v>317</v>
       </c>
+      <c r="F52" s="139"/>
+      <c r="G52" s="139"/>
+      <c r="H52" s="139" t="s">
+        <v>343</v>
+      </c>
     </row>
-    <row r="53" spans="1:2" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:8" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A53" s="135" t="s">
         <v>40</v>
       </c>
       <c r="B53" s="5" t="s">
         <v>318</v>
       </c>
+      <c r="F53" s="139"/>
+      <c r="G53" s="139"/>
+      <c r="H53" s="139" t="s">
+        <v>343</v>
+      </c>
     </row>
-    <row r="54" spans="1:2" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:8" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A54" s="132" t="s">
         <v>47</v>
       </c>
       <c r="B54" s="5" t="s">
         <v>319</v>
       </c>
+      <c r="F54" s="139"/>
+      <c r="G54" s="139"/>
+      <c r="H54" s="139" t="s">
+        <v>343</v>
+      </c>
     </row>
-    <row r="55" spans="1:2" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:8" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A55" s="133" t="s">
         <v>48</v>
       </c>
       <c r="B55" s="5" t="s">
         <v>320</v>
       </c>
+      <c r="F55" s="139"/>
+      <c r="G55" s="139"/>
+      <c r="H55" s="139" t="s">
+        <v>343</v>
+      </c>
     </row>
-    <row r="56" spans="1:2" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:8" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A56" s="135" t="s">
         <v>49</v>
       </c>
       <c r="B56" s="5" t="s">
         <v>321</v>
       </c>
+      <c r="F56" s="139"/>
+      <c r="G56" s="139"/>
+      <c r="H56" s="139" t="s">
+        <v>343</v>
+      </c>
     </row>
-    <row r="57" spans="1:2" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:8" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A57" s="132" t="s">
         <v>50</v>
       </c>
       <c r="B57" s="5" t="s">
         <v>322</v>
       </c>
+      <c r="F57" s="139"/>
+      <c r="G57" s="139"/>
+      <c r="H57" s="139" t="s">
+        <v>343</v>
+      </c>
     </row>
-    <row r="58" spans="1:2" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:8" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A58" s="133" t="s">
         <v>51</v>
       </c>
       <c r="B58" s="5" t="s">
         <v>323</v>
       </c>
+      <c r="F58" s="139"/>
+      <c r="G58" s="139"/>
+      <c r="H58" s="139" t="s">
+        <v>343</v>
+      </c>
     </row>
-    <row r="59" spans="1:2" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:8" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A59" s="135" t="s">
         <v>52</v>
       </c>
       <c r="B59" s="5" t="s">
         <v>324</v>
       </c>
+      <c r="F59" s="139"/>
+      <c r="G59" s="139"/>
+      <c r="H59" s="139" t="s">
+        <v>343</v>
+      </c>
     </row>
-    <row r="60" spans="1:2" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:8" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A60" s="132" t="s">
         <v>53</v>
       </c>
       <c r="B60" s="5" t="s">
         <v>325</v>
       </c>
+      <c r="F60" s="139"/>
+      <c r="G60" s="139"/>
+      <c r="H60" s="139" t="s">
+        <v>343</v>
+      </c>
     </row>
-    <row r="61" spans="1:2" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:8" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A61" s="133" t="s">
         <v>54</v>
       </c>
       <c r="B61" s="5" t="s">
         <v>326</v>
       </c>
+      <c r="F61" s="139"/>
+      <c r="G61" s="139"/>
+      <c r="H61" s="139" t="s">
+        <v>343</v>
+      </c>
     </row>
-    <row r="62" spans="1:2" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:8" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A62" s="130" t="s">
         <v>55</v>
       </c>
       <c r="B62" s="5" t="s">
         <v>327</v>
       </c>
+      <c r="F62" s="140"/>
+      <c r="G62" s="140"/>
+      <c r="H62" s="140" t="s">
+        <v>346</v>
+      </c>
     </row>
-    <row r="63" spans="1:2" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:8" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A63" s="130" t="s">
         <v>56</v>
       </c>
       <c r="B63" s="5" t="s">
         <v>328</v>
       </c>
+      <c r="F63" s="140"/>
+      <c r="G63" s="140"/>
+      <c r="H63" s="140" t="s">
+        <v>346</v>
+      </c>
     </row>
-    <row r="64" spans="1:2" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:8" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A64" s="132" t="s">
         <v>57</v>
       </c>
       <c r="B64" s="5" t="s">
         <v>329</v>
       </c>
+      <c r="F64" s="140"/>
+      <c r="G64" s="140"/>
+      <c r="H64" s="140" t="s">
+        <v>346</v>
+      </c>
     </row>
-    <row r="65" spans="1:2" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:8" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A65" s="130" t="s">
         <v>58</v>
       </c>
       <c r="B65" s="5" t="s">
         <v>330</v>
       </c>
+      <c r="F65" s="138"/>
+      <c r="G65" s="138"/>
+      <c r="H65" s="138" t="s">
+        <v>344</v>
+      </c>
     </row>
-    <row r="66" spans="1:2" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:8" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A66" s="130" t="s">
         <v>59</v>
       </c>
       <c r="B66" s="5" t="s">
         <v>331</v>
       </c>
+      <c r="F66" s="138"/>
+      <c r="G66" s="138"/>
+      <c r="H66" s="138" t="s">
+        <v>344</v>
+      </c>
     </row>
-    <row r="67" spans="1:2" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:8" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A67" s="132" t="s">
         <v>60</v>
       </c>
       <c r="B67" s="5" t="s">
         <v>332</v>
       </c>
+      <c r="F67" s="138"/>
+      <c r="G67" s="138"/>
+      <c r="H67" s="138" t="s">
+        <v>344</v>
+      </c>
     </row>
-    <row r="68" spans="1:2" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:8" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A68" s="130" t="s">
         <v>61</v>
       </c>
       <c r="B68" s="5" t="s">
         <v>333</v>
       </c>
+      <c r="F68" s="140"/>
+      <c r="G68" s="140"/>
+      <c r="H68" s="140" t="s">
+        <v>346</v>
+      </c>
     </row>
-    <row r="69" spans="1:2" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:8" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A69" s="130" t="s">
         <v>62</v>
       </c>
       <c r="B69" s="5" t="s">
         <v>334</v>
       </c>
+      <c r="F69" s="139"/>
+      <c r="G69" s="139"/>
+      <c r="H69" s="139" t="s">
+        <v>343</v>
+      </c>
     </row>
-    <row r="70" spans="1:2" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:8" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A70" s="132" t="s">
         <v>63</v>
       </c>
       <c r="B70" s="5" t="s">
         <v>335</v>
       </c>
+      <c r="F70" s="140"/>
+      <c r="G70" s="140"/>
+      <c r="H70" s="140" t="s">
+        <v>346</v>
+      </c>
     </row>
-    <row r="71" spans="1:2" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:8" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A71" s="133" t="s">
         <v>64</v>
       </c>
       <c r="B71" s="5" t="s">
         <v>336</v>
       </c>
+      <c r="F71" s="141"/>
+      <c r="G71" s="141"/>
+      <c r="H71" s="141" t="s">
+        <v>347</v>
+      </c>
     </row>
-    <row r="72" spans="1:2" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:8" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A72" s="133" t="s">
         <v>65</v>
       </c>
       <c r="B72" s="5" t="s">
         <v>337</v>
       </c>
+      <c r="F72" s="141"/>
+      <c r="G72" s="141"/>
+      <c r="H72" s="141" t="s">
+        <v>347</v>
+      </c>
     </row>
-    <row r="73" spans="1:2" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:8" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A73" s="130" t="s">
         <v>66</v>
       </c>
       <c r="B73" s="5" t="s">
         <v>338</v>
       </c>
+      <c r="F73" s="139"/>
+      <c r="G73" s="139"/>
+      <c r="H73" s="139" t="s">
+        <v>343</v>
+      </c>
     </row>
-    <row r="74" spans="1:2" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:8" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A74" s="130" t="s">
         <v>67</v>
       </c>
       <c r="B74" s="5" t="s">
         <v>339</v>
       </c>
+      <c r="F74" s="139"/>
+      <c r="G74" s="139"/>
+      <c r="H74" s="139" t="s">
+        <v>343</v>
+      </c>
     </row>
-    <row r="75" spans="1:2" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:8" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A75" s="130" t="s">
         <v>68</v>
       </c>
       <c r="B75" s="5" t="s">
         <v>340</v>
       </c>
+      <c r="F75" s="139"/>
+      <c r="G75" s="139"/>
+      <c r="H75" s="139" t="s">
+        <v>343</v>
+      </c>
     </row>
-    <row r="76" spans="1:2" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:8" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A76" s="130" t="s">
         <v>69</v>
       </c>
       <c r="B76" s="5" t="s">
         <v>341</v>
+      </c>
+      <c r="F76" s="138"/>
+      <c r="G76" s="138"/>
+      <c r="H76" s="138" t="s">
+        <v>344</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Moved where some markdowns are located.
</commit_message>
<xml_diff>
--- a/UW_Nest_Behavioral_Sheets_Cleaned.xlsx
+++ b/UW_Nest_Behavioral_Sheets_Cleaned.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jacobchung/coding_projects/Owrasse_Underwater_Behavioral_Sheet/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{997F1C79-08CD-5947-BC14-AFC7DE4D7B69}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8CC1BF81-6568-6046-921D-8607D8A090BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-20" yWindow="520" windowWidth="27760" windowHeight="17500" xr2:uid="{F3336806-D2AA-0243-9E92-F92A9E05C0A5}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="27760" windowHeight="17500" activeTab="1" xr2:uid="{F3336806-D2AA-0243-9E92-F92A9E05C0A5}"/>
   </bookViews>
   <sheets>
     <sheet name="UW_Behavior_Sheets" sheetId="1" r:id="rId1"/>

</xml_diff>